<commit_message>
Mark 4 leads as confirmed No via override
Rubio Attorneys, Pathlight Legal, SLC Law Office, Wattel & York confirmed
declined by rep; override estimate to No across reports, action plan, and
re-engagement audience (now 207 leads). Refresh sequence doc counts.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0188Gg43mP68tZqBh1g3KVvC
</commit_message>
<xml_diff>
--- a/MBP_Follow_Up_Report__Current.xlsx
+++ b/MBP_Follow_Up_Report__Current.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Follow-Up Report" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Legend &amp; Method" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Follow-Up Report" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend &amp; Method" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Follow-Up Report'!$A$4:$K$299</definedName>
@@ -7689,14 +7689,14 @@
           <t>Had Meeting</t>
         </is>
       </c>
-      <c r="I146" s="11" t="inlineStr">
-        <is>
-          <t>Maybe Later</t>
+      <c r="I146" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
       <c r="J146" s="8" t="inlineStr">
         <is>
-          <t>Had the meeting; no signed decision yet. Following up to move it forward — still in play.</t>
+          <t>Followed up after earlier interest; they confirmed they are not moving forward — declined.</t>
         </is>
       </c>
       <c r="K146" s="7" t="inlineStr"/>
@@ -8265,14 +8265,14 @@
           <t>Had Meeting</t>
         </is>
       </c>
-      <c r="I158" s="11" t="inlineStr">
-        <is>
-          <t>Maybe Later</t>
+      <c r="I158" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
       <c r="J158" s="8" t="inlineStr">
         <is>
-          <t>Had the meeting; no signed decision yet. Following up to move it forward — still in play.</t>
+          <t>Followed up after earlier interest; they confirmed they are not moving forward — declined.</t>
         </is>
       </c>
       <c r="K158" s="7" t="inlineStr"/>
@@ -8731,14 +8731,14 @@
           <t>Had Meeting</t>
         </is>
       </c>
-      <c r="I168" s="11" t="inlineStr">
-        <is>
-          <t>Maybe Later</t>
+      <c r="I168" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
       <c r="J168" s="8" t="inlineStr">
         <is>
-          <t>Had the meeting; no signed decision yet. Following up to move it forward — still in play.</t>
+          <t>Followed up after earlier interest; they confirmed they are not moving forward — declined.</t>
         </is>
       </c>
       <c r="K168" s="7" t="inlineStr"/>
@@ -12679,14 +12679,14 @@
           <t>Interested</t>
         </is>
       </c>
-      <c r="I252" s="11" t="inlineStr">
-        <is>
-          <t>Maybe Later</t>
+      <c r="I252" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
       <c r="J252" s="8" t="inlineStr">
         <is>
-          <t>Replied positively and asked for a meeting; following up to lock in a time — open, warm lead.</t>
+          <t>Followed up after earlier interest; they confirmed they are not moving forward — declined.</t>
         </is>
       </c>
       <c r="K252" s="7" t="inlineStr"/>
@@ -14746,11 +14746,11 @@
         </is>
       </c>
       <c r="B5" s="14" t="n">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>28.1%</t>
+          <t>26.8%</t>
         </is>
       </c>
     </row>
@@ -14776,11 +14776,11 @@
         </is>
       </c>
       <c r="B7" s="14" t="n">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C7" s="14" t="inlineStr">
         <is>
-          <t>14.6%</t>
+          <t>15.9%</t>
         </is>
       </c>
     </row>
@@ -14845,7 +14845,7 @@
         </is>
       </c>
       <c r="B14" s="22" t="n">
-        <v>83</v>
+        <v>79</v>
       </c>
     </row>
     <row r="15">
@@ -14855,7 +14855,7 @@
         </is>
       </c>
       <c r="B15" s="22" t="n">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="16">

</xml_diff>